<commit_message>
V1.1 simplification pass: remove AI scoring, Every Lead Alert, email-first reporting
Remove AI lead scoring (Lead Score/Temperature/Urgency, Sonnet 4.6) system-wide;
rename "Hot Lead Alert" to "Every Lead Alert" (workflow 04) so every submission
triggers the owner alert via email by default (SMS built but disabled, toggled
per client). Convert internal reporting (07/08/11/12) from SMS-only to
email-first via a shared CONFIG block, professionalize lead-notification emails,
overhaul appointment scheduling to a structured date/time picker with
configurable business hours (workflow 06), and standardize all timestamps to
America/New_York via Luxon. Simplify the Leads CRM tab from 20 to 17 columns,
update the CRM template, and reconcile all affected docs and founder playbooks.
Add docs/V1_1_RECONCILIATION.md as the canonical changelog for this pass.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/templates/Roofing_CRM_Google_Sheets_TEMPLATE.xlsx
+++ b/templates/Roofing_CRM_Google_Sheets_TEMPLATE.xlsx
@@ -73,7 +73,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -81,6 +81,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -446,7 +447,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T5"/>
+  <dimension ref="A1:Q5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -461,14 +462,11 @@
     <col width="32" customWidth="1" min="10" max="10"/>
     <col width="14" customWidth="1" min="11" max="11"/>
     <col width="16" customWidth="1" min="12" max="12"/>
-    <col width="10" customWidth="1" min="13" max="13"/>
-    <col width="12" customWidth="1" min="14" max="14"/>
-    <col width="12" customWidth="1" min="15" max="15"/>
+    <col width="12" customWidth="1" min="13" max="13"/>
+    <col width="18" customWidth="1" min="14" max="14"/>
+    <col width="14" customWidth="1" min="15" max="15"/>
     <col width="12" customWidth="1" min="16" max="16"/>
-    <col width="18" customWidth="1" min="17" max="17"/>
-    <col width="14" customWidth="1" min="18" max="18"/>
-    <col width="12" customWidth="1" min="19" max="19"/>
-    <col width="40" customWidth="1" min="20" max="20"/>
+    <col width="40" customWidth="1" min="17" max="17"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -534,40 +532,25 @@
       </c>
       <c r="M1" s="1" t="inlineStr">
         <is>
-          <t>Lead Score</t>
+          <t>Status</t>
         </is>
       </c>
       <c r="N1" s="1" t="inlineStr">
         <is>
-          <t>Temperature</t>
+          <t>Last Contact</t>
         </is>
       </c>
       <c r="O1" s="1" t="inlineStr">
         <is>
-          <t>Urgency</t>
+          <t>Follow-up Count</t>
         </is>
       </c>
       <c r="P1" s="1" t="inlineStr">
         <is>
-          <t>Status</t>
+          <t>Assigned To</t>
         </is>
       </c>
       <c r="Q1" s="1" t="inlineStr">
-        <is>
-          <t>Last Contact</t>
-        </is>
-      </c>
-      <c r="R1" s="1" t="inlineStr">
-        <is>
-          <t>Follow-up Count</t>
-        </is>
-      </c>
-      <c r="S1" s="1" t="inlineStr">
-        <is>
-          <t>Assigned To</t>
-        </is>
-      </c>
-      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
@@ -581,7 +564,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>2026-06-01T09:14:00Z</t>
+          <t>2026-06-01T09:14:00.000-04:00</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
@@ -630,40 +613,27 @@
           <t>Weekday mornings</t>
         </is>
       </c>
-      <c r="M2" s="2" t="n">
-        <v>86</v>
+      <c r="M2" s="2" t="inlineStr">
+        <is>
+          <t>Booked</t>
+        </is>
       </c>
       <c r="N2" s="2" t="inlineStr">
         <is>
-          <t>Hot</t>
-        </is>
-      </c>
-      <c r="O2" s="2" t="inlineStr">
-        <is>
-          <t>Emergency</t>
-        </is>
+          <t>2026-06-01T09:20:00.000-04:00</t>
+        </is>
+      </c>
+      <c r="O2" s="2" t="n">
+        <v>1</v>
       </c>
       <c r="P2" s="2" t="inlineStr">
         <is>
-          <t>Booked</t>
+          <t>J. Reyes</t>
         </is>
       </c>
       <c r="Q2" s="2" t="inlineStr">
         <is>
-          <t>2026-06-01T09:20:00Z</t>
-        </is>
-      </c>
-      <c r="R2" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="S2" s="2" t="inlineStr">
-        <is>
-          <t>J. Reyes</t>
-        </is>
-      </c>
-      <c r="T2" s="2" t="inlineStr">
-        <is>
-          <t>Example row — replace with real data. Active leak, scored Hot/Emergency by AI scoring (workflow 02).</t>
+          <t>Example row — replace with real data.</t>
         </is>
       </c>
     </row>
@@ -675,7 +645,7 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-02T14:02:00Z</t>
+          <t>2026-06-02T14:02:00.000-04:00</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
@@ -704,24 +674,17 @@
       <c r="J3" s="2" t="inlineStr"/>
       <c r="K3" s="2" t="inlineStr"/>
       <c r="L3" s="2" t="inlineStr"/>
-      <c r="M3" s="2" t="inlineStr"/>
-      <c r="N3" s="2" t="inlineStr">
-        <is>
-          <t>Cold</t>
-        </is>
-      </c>
-      <c r="O3" s="2" t="inlineStr"/>
-      <c r="P3" s="2" t="inlineStr">
+      <c r="M3" s="2" t="inlineStr">
         <is>
           <t>New</t>
         </is>
       </c>
-      <c r="Q3" s="2" t="inlineStr"/>
-      <c r="R3" s="2" t="n">
+      <c r="N3" s="2" t="inlineStr"/>
+      <c r="O3" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="S3" s="2" t="inlineStr"/>
-      <c r="T3" s="2" t="inlineStr">
+      <c r="P3" s="2" t="inlineStr"/>
+      <c r="Q3" s="2" t="inlineStr">
         <is>
           <t>Example row — missed-call auto-SMS sent (workflow 03); no Lead record is normally created for pure missed calls — this row illustrates what a follow-up form submission from the same number would look like once captured.</t>
         </is>
@@ -730,13 +693,13 @@
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>SOURCE OF TRUTH: matches the live CRM Adapter sub-workflow contract exactly (workflow 01, id wVRHChyFrUNRaH4M) — verified against production data. 'Lead ID' and 'Phone' are the match keys; new leads get LEAD-#### minted by the adapter. Do not rename/remove columns — every workflow that scores, follows up, reminds, or reports on leads depends on these exact header names.</t>
+          <t>SOURCE OF TRUTH: matches the live CRM Adapter sub-workflow contract exactly (workflow 01, id wVRHChyFrUNRaH4M) — verified against production data. 'Lead ID' and 'Phone' are the match keys; new leads get LEAD-#### minted by the adapter. Do not rename/remove columns — every workflow that follows up, reminds, or reports on leads depends on these exact header names. V1.1 (2026-06-11): 'Lead Score', 'Temperature', and 'Urgency' columns were removed system-wide — AI lead scoring was removed; every lead now follows the same 'Every Lead Alert' notification path (see docs/V1_1_RECONCILIATION.md). All timestamps are ISO 8601 in America/New_York (Boston time), the system-wide default timezone.</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A5:T5"/>
+    <mergeCell ref="A5:Q5"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1629,7 +1592,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C9"/>
+  <dimension ref="A1:C8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -1665,7 +1628,7 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>PLACEHOLDER — replace with e.g. =COUNTIFS(Leads!P:P,"&lt;&gt;Booked",Leads!P:P,"&lt;&gt;Lost") once real data exists.</t>
+          <t>PLACEHOLDER — replace with e.g. =COUNTIFS(Leads!M:M,"&lt;&gt;Booked",Leads!M:M,"&lt;&gt;Lost") once real data exists. ('Status' is column M in the V1.1 17-column Leads schema.)</t>
         </is>
       </c>
     </row>
@@ -1687,7 +1650,7 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Hot/Emergency Leads (Open)</t>
+          <t>Appointments This Week</t>
         </is>
       </c>
       <c r="B4" s="4" t="n">
@@ -1695,14 +1658,14 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>PLACEHOLDER — e.g. =COUNTIFS(Leads!N:N,"Hot",Leads!P:P,"&lt;&gt;Booked")  (combine with an OR for Urgency="Emergency" via SUMPRODUCT if needed)</t>
+          <t>PLACEHOLDER — e.g. =COUNTIFS(Appointments!G:G, "&gt;="&amp;TEXT(TODAY()-7,"YYYY-MM-DD"))</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Appointments This Week</t>
+          <t>Jobs Completed This Month</t>
         </is>
       </c>
       <c r="B5" s="4" t="n">
@@ -1710,14 +1673,14 @@
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>PLACEHOLDER — e.g. =COUNTIFS(Appointments!G:G, "&gt;="&amp;TEXT(TODAY()-7,"YYYY-MM-DD"))</t>
+          <t>PLACEHOLDER — depends on the Jobs tab going live first (see that tab's note); e.g. =COUNTIFS(Jobs!I:I,"Completed",Jobs!K:K,"&gt;="&amp;EOMONTH(TODAY(),-1)+1)</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Jobs Completed This Month</t>
+          <t>Stale Leads (No Contact 7+ Days)</t>
         </is>
       </c>
       <c r="B6" s="4" t="n">
@@ -1725,35 +1688,23 @@
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>PLACEHOLDER — depends on the Jobs tab going live first (see that tab's note); e.g. =COUNTIFS(Jobs!I:I,"Completed",Jobs!K:K,"&gt;="&amp;EOMONTH(TODAY(),-1)+1)</t>
+          <t>PLACEHOLDER — mirrors workflow 07's own 'Stale' definition; e.g. =COUNTIFS(Leads!N:N,"&lt;"&amp;TEXT(TODAY()-7,"YYYY-MM-DD"))  — keep this formula in sync with whatever workflow 07 (Pipeline Status Digest) uses internally so the dashboard never disagrees with its email digest. ('Last Contact' is column N in the V1.1 17-column Leads schema.)</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="2" t="inlineStr">
-        <is>
-          <t>Stale Leads (No Contact 7+ Days)</t>
-        </is>
-      </c>
-      <c r="B7" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="C7" s="2" t="inlineStr">
-        <is>
-          <t>PLACEHOLDER — mirrors workflow 07's own 'Stale' definition; e.g. =COUNTIFS(Leads!Q:Q,"&lt;"&amp;TEXT(TODAY()-7,"YYYY-MM-DD"))  — keep this formula in sync with whatever workflow 07 (Pipeline Status Digest) uses internally so the dashboard never disagrees with the SMS digest</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="3" t="inlineStr">
-        <is>
-          <t>⚠️ THIS TAB IS A SUMMARY VIEW, NOT A DATA-ENTRY TAB — it is meant to hold live formulas that reference the other tabs, not raw rows. No workflow currently writes to or reads from it; the system's owner-facing reporting is delivered instead via SMS digests (workflows 07/08) and (as of 2026-06-07) Workflow 11's health alerts. The 'Value' column above is intentionally left at 0/placeholder — replace each with a live formula (see the Notes column for a starting point per metric) once the sheet has real rows to compute against. Keep every formula's definition of a status ('Stale', 'Hot', etc.) in sync with the corresponding live workflow's own definition — a Dashboard that disagrees with the SMS digest the owner already trusts is worse than no Dashboard at all.</t>
+      <c r="B7" s="5" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>⚠️ THIS TAB IS A SUMMARY VIEW, NOT A DATA-ENTRY TAB — it is meant to hold live formulas that reference the other tabs, not raw rows. No workflow currently writes to or reads from it; the system's owner-facing reporting is delivered instead via email digests (workflows 07/08, converted from SMS to email in V1.1) and Workflow 11's health alerts. The 'Value' column above is intentionally left at 0/placeholder — replace each with a live formula (see the Notes column for a starting point per metric) once the sheet has real rows to compute against. Keep every formula's definition of a status ('Stale', etc.) in sync with the corresponding live workflow's own definition — a Dashboard that disagrees with the email digest the owner already trusts is worse than no Dashboard at all. V1.1 (2026-06-11): the 'Hot/Emergency Leads (Open)' metric was removed along with AI lead scoring system-wide.</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A9:C9"/>
+    <mergeCell ref="A8:C8"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add Workflow 13: Appointment Reschedule Notifier (V1.1 reconciliation fix)
Closes a real QA-discovered gap: when the owner manually moves a
Scheduled appointment after the customer was already notified, the
customer previously received no follow-up. Workflow 13 detects the
mismatch between Appt Date/Time and the new Notified Appt Date/Time
columns, texts the customer the new time, emails the owner, resets
the 24h/2h reminder flags so Workflow 09 sends fresh reminders, and
logs the SMS via the CRM Adapter. Idempotent by design.

Workflow 06 now seeds Notified Appt Date/Time at booking time.
Docs, CRM schema, and the CRM template updated to reflect the new
17-column Appointments schema and the 13-workflow inventory.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/templates/Roofing_CRM_Google_Sheets_TEMPLATE.xlsx
+++ b/templates/Roofing_CRM_Google_Sheets_TEMPLATE.xlsx
@@ -711,7 +711,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O4"/>
+  <dimension ref="A1:Q4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -729,6 +729,8 @@
     <col width="14" customWidth="1" min="13" max="13"/>
     <col width="12" customWidth="1" min="14" max="14"/>
     <col width="40" customWidth="1" min="15" max="15"/>
+    <col width="18" customWidth="1" min="16" max="16"/>
+    <col width="18" customWidth="1" min="17" max="17"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -805,6 +807,16 @@
       <c r="O1" s="1" t="inlineStr">
         <is>
           <t>Notes</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>Notified Appt Date</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>Notified Appt Time</t>
         </is>
       </c>
     </row>
@@ -868,17 +880,27 @@
           <t>Example row — booked via owner-facing form (workflow 06).</t>
         </is>
       </c>
+      <c r="P2" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-10</t>
+        </is>
+      </c>
+      <c r="Q2" s="2" t="inlineStr">
+        <is>
+          <t>10:00 AM</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>SOURCE OF TRUTH: matches the exact column set written by workflow 06's 'Write Appointment' node (live, verified) — 15 columns. 'Appt Date' must stay 'YYYY-MM-DD' and 'Appt Time' must stay 'H:MM AM/PM' — both workflow 09 (Reminders) and workflow 11 (Health Monitor) parse these with strict regexes. 'Reminder 24h'/'Reminder 2h' are write-only flag columns — leave them blank; the system manages them. 'Team Approval' and 'Calendar Event ID' are reserved for future phases (crew-approval workflow, calendar sync) — currently always blank.</t>
+          <t>SOURCE OF TRUTH: matches the exact column set written by workflow 06's 'Write Appointment' node (live, verified) — 17 columns. 'Appt Date' must stay 'YYYY-MM-DD' and 'Appt Time' must stay 'H:MM AM/PM' — workflows 09 (Reminders), 11 (Health Monitor), and 13 (Reschedule Notifier) parse these with strict regexes. 'Reminder 24h'/'Reminder 2h' are write-only flag columns — leave them blank; the system manages them. 'Team Approval' and 'Calendar Event ID' are reserved for future phases (crew-approval workflow, calendar sync) — currently always blank. 'Notified Appt Date'/'Notified Appt Time' (added 2026-06-12) should be seeded equal to 'Appt Date'/'Appt Time' at booking time — workflow 13 compares against these to detect owner-initiated reschedules and notify the customer.</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A4:O4"/>
+    <mergeCell ref="A4:Q4"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Convert Notify Customer to a Send Update/No dropdown across WF13, CRM template, and docs
Replaces the typed TRUE/FALSE Notify Customer field with a strict
"No"/"Send Update" dropdown (matching live Appointments sheet styling),
defaulting to "No". WF13 triggers on "Send Update" and resets the field
back to "No" after a successful reschedule notification, preserving the
YES/NO confirmation flow and two-attempt escalation rule.
</commit_message>
<xml_diff>
--- a/templates/Roofing_CRM_Google_Sheets_TEMPLATE.xlsx
+++ b/templates/Roofing_CRM_Google_Sheets_TEMPLATE.xlsx
@@ -711,7 +711,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q4"/>
+  <dimension ref="A1:T4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -731,6 +731,9 @@
     <col width="40" customWidth="1" min="15" max="15"/>
     <col width="18" customWidth="1" min="16" max="16"/>
     <col width="18" customWidth="1" min="17" max="17"/>
+    <col width="16" customWidth="1" min="18" max="18"/>
+    <col width="16" customWidth="1" min="19" max="19"/>
+    <col width="16" customWidth="1" min="20" max="20"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -817,6 +820,21 @@
       <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>Notified Appt Time</t>
+        </is>
+      </c>
+      <c r="R1" s="1" t="inlineStr">
+        <is>
+          <t>Notify Customer</t>
+        </is>
+      </c>
+      <c r="S1" s="1" t="inlineStr">
+        <is>
+          <t>Reschedule Status</t>
+        </is>
+      </c>
+      <c r="T1" s="1" t="inlineStr">
+        <is>
+          <t>Reschedule Attempts</t>
         </is>
       </c>
     </row>
@@ -890,18 +908,36 @@
           <t>10:00 AM</t>
         </is>
       </c>
+      <c r="R2" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="S2" s="2" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="T2" s="2" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>SOURCE OF TRUTH: matches the exact column set written by workflow 06's 'Write Appointment' node (live, verified) — 17 columns. 'Appt Date' must stay 'YYYY-MM-DD' and 'Appt Time' must stay 'H:MM AM/PM' — workflows 09 (Reminders), 11 (Health Monitor), and 13 (Reschedule Notifier) parse these with strict regexes. 'Reminder 24h'/'Reminder 2h' are write-only flag columns — leave them blank; the system manages them. 'Team Approval' and 'Calendar Event ID' are reserved for future phases (crew-approval workflow, calendar sync) — currently always blank. 'Notified Appt Date'/'Notified Appt Time' (added 2026-06-12) should be seeded equal to 'Appt Date'/'Appt Time' at booking time — workflow 13 compares against these to detect owner-initiated reschedules and notify the customer.</t>
+          <t>SOURCE OF TRUTH: matches the exact column set written by workflow 06's 'Write Appointment' node (live, verified) — 20 columns. 'Appt Date' must stay 'YYYY-MM-DD' and 'Appt Time' must stay 'H:MM AM/PM' — workflows 09 (Reminders), 11 (Health Monitor), and 13 (Reschedule Notifier) parse these with strict regexes. 'Reminder 24h'/'Reminder 2h' are write-only flag columns — leave them blank; the system manages them. 'Team Approval' and 'Calendar Event ID' are reserved for future phases (crew-approval workflow, calendar sync) — currently always blank. 'Notified Appt Date'/'Notified Appt Time' (added 2026-06-12) should be seeded equal to 'Appt Date'/'Appt Time' at booking time — workflow 13 compares against these to detect owner-initiated reschedules and notify the customer. 'Notify Customer' (added 2026-06-13) is a dropdown defaulting to 'No' — the owner picks 'Send Update' to trigger workflow 13's reschedule-notification flow; workflow 13 resets it back to 'No' after a successful run so the field can be reused for another notification later. 'Reschedule Status' ('None'/'Pending Customer Confirmation'/'Confirmed'/'Escalated to Owner') and 'Reschedule Attempts' (0-2) track the YES/NO customer-confirmation flow and the two-attempt escalation rule — both managed by workflow 13 and reset to 'None'/0 on each new notification cycle.</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A4:Q4"/>
+    <mergeCell ref="A4:T4"/>
   </mergeCells>
+  <dataValidations count="1">
+    <dataValidation sqref="R2:R200" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" errorTitle="Invalid entry" error="Please select 'No' or 'Send Update' from the dropdown." type="list" errorStyle="stop">
+      <formula1>"No,Send Update"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>